<commit_message>
docs: refresh official submission artifacts
</commit_message>
<xml_diff>
--- a/outputs/hw06/HW06_Test_Cases.xlsx
+++ b/outputs/hw06/HW06_Test_Cases.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R230d5d5454954b64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="R55cb26099831420f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="Rf991ddaec7e84db0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="R49048ed3a2834e31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="R8654984d71494f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="Rebccac0424004c84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="Rbeca8c3e8d184c2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R31dc64276ff34331"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="Rd508a98d75b042f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="Rd9aab81921e84b0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="R65c0221703344d51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="Rb379b6e4ba3248d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="R8c28afe74a5a4bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="R5a05c2aa6fcf45a9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -239,7 +239,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="22">
+  <x:dxfs count="23">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -441,6 +441,17 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF067647"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFEAF8F0"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
@@ -498,7 +509,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>Dry-run pass/fail by API</a:t>
+              <a:t>Official pass/fail by API</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -650,7 +661,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rce8f746b67f845d5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1cc720a8b94c496b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -673,8 +684,8 @@
     <x:tableColumn id="9" name="Oracle"/>
     <x:tableColumn id="10" name="Input / mode"/>
     <x:tableColumn id="11" name="Manual_Review"/>
-    <x:tableColumn id="12" name="Dry_Result"/>
-    <x:tableColumn id="13" name="Dry_Failures"/>
+    <x:tableColumn id="12" name="Official_Result"/>
+    <x:tableColumn id="13" name="Official_Failures"/>
     <x:tableColumn id="14" name="Human_Verified"/>
     <x:tableColumn id="15" name="Reviewer_Notes"/>
   </x:tableColumns>
@@ -696,8 +707,8 @@
     <x:tableColumn id="9" name="Oracle"/>
     <x:tableColumn id="10" name="Input / mode"/>
     <x:tableColumn id="11" name="Manual_Review"/>
-    <x:tableColumn id="12" name="Dry_Result"/>
-    <x:tableColumn id="13" name="Dry_Failures"/>
+    <x:tableColumn id="12" name="Official_Result"/>
+    <x:tableColumn id="13" name="Official_Failures"/>
     <x:tableColumn id="14" name="Human_Verified"/>
     <x:tableColumn id="15" name="Reviewer_Notes"/>
   </x:tableColumns>
@@ -719,8 +730,8 @@
     <x:tableColumn id="9" name="Oracle"/>
     <x:tableColumn id="10" name="Input / mode"/>
     <x:tableColumn id="11" name="Manual_Review"/>
-    <x:tableColumn id="12" name="Dry_Result"/>
-    <x:tableColumn id="13" name="Dry_Failures"/>
+    <x:tableColumn id="12" name="Official_Result"/>
+    <x:tableColumn id="13" name="Official_Failures"/>
     <x:tableColumn id="14" name="Human_Verified"/>
     <x:tableColumn id="15" name="Reviewer_Notes"/>
   </x:tableColumns>
@@ -743,14 +754,15 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="BugSummaryTable" displayName="BugSummaryTable" ref="A4:F14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="BugSummaryTable" displayName="BugSummaryTable" ref="A4:G14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="Bug_ID"/>
     <x:tableColumn id="2" name="Severity"/>
     <x:tableColumn id="3" name="Area"/>
     <x:tableColumn id="4" name="Finding"/>
     <x:tableColumn id="5" name="Evidence"/>
     <x:tableColumn id="6" name="GitHub_Status"/>
+    <x:tableColumn id="7" name="Issue_URL"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -978,7 +990,7 @@
     <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="4" t="str">
         <x:v>HW06 API Testing Dashboard
-Formula-backed summary • Hưng Nguyễn • Student ID HUMAN_REVIEW_REQUIRED</x:v>
+Formula-backed summary • Nguyễn Đình Thái Hưng • Student ID 23127373</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -1225,11 +1237,11 @@
         <x:v>Student ID supplied</x:v>
       </x:c>
       <x:c r="B12" s="42" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="C12" s="37"/>
       <x:c r="D12" s="37" t="str">
-        <x:v>Dry-run total</x:v>
+        <x:v>Official total</x:v>
       </x:c>
       <x:c r="E12" s="37" t="n">
         <x:v>158</x:v>
@@ -1246,11 +1258,11 @@
         <x:v>Official Newman rerun</x:v>
       </x:c>
       <x:c r="B13" s="42" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="C13" s="37"/>
       <x:c r="D13" s="37" t="str">
-        <x:v>Dry-run passed</x:v>
+        <x:v>Official passed</x:v>
       </x:c>
       <x:c r="E13" s="37" t="n">
         <x:v>113</x:v>
@@ -1271,7 +1283,7 @@
       </x:c>
       <x:c r="C14" s="37"/>
       <x:c r="D14" s="37" t="str">
-        <x:v>Dry-run failed</x:v>
+        <x:v>Official failed</x:v>
       </x:c>
       <x:c r="E14" s="37" t="n">
         <x:v>45</x:v>
@@ -1292,13 +1304,13 @@
       </x:c>
       <x:c r="C15" s="37"/>
       <x:c r="D15" s="37" t="str">
-        <x:v>Bug candidates</x:v>
+        <x:v>GitHub Issues</x:v>
       </x:c>
       <x:c r="E15" s="37" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="37" t="str">
-        <x:v>Needs GitHub publication</x:v>
+        <x:v>10 expected</x:v>
       </x:c>
       <x:c r="G15" s="37"/>
       <x:c r="H15" s="37"/>
@@ -1306,7 +1318,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="37" t="str">
-        <x:v>Public GitHub + issues</x:v>
+        <x:v>Ten GitHub Issues</x:v>
       </x:c>
       <x:c r="B16" s="42" t="str">
         <x:v>NO</x:v>
@@ -1327,7 +1339,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="37" t="str">
-        <x:v>Video + final ZIP</x:v>
+        <x:v>Public GitHub</x:v>
       </x:c>
       <x:c r="B17" s="42" t="str">
         <x:v>NO</x:v>
@@ -1340,6 +1352,21 @@
       <x:c r="H17" s="37"/>
       <x:c r="I17" s="37"/>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="37" t="str">
+        <x:v>Video + final ZIP</x:v>
+      </x:c>
+      <x:c r="B18" s="42" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="C18" s="37"/>
+      <x:c r="D18" s="37"/>
+      <x:c r="E18" s="37"/>
+      <x:c r="F18" s="37"/>
+      <x:c r="G18" s="37"/>
+      <x:c r="H18" s="37"/>
+      <x:c r="I18" s="37"/>
+    </x:row>
     <x:row r="20">
       <x:c r="K20" t="str">
         <x:v>API</x:v>
@@ -1394,8 +1421,11 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:I2"/>
   </x:mergeCells>
+  <x:conditionalFormatting sqref="B12:B18">
+    <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="YES"/>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ea5ae5fff84162"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64ced6bb13b74d5f"/>
 </x:worksheet>
 </file>
 
@@ -1423,7 +1453,7 @@
     <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="4" t="str">
         <x:v>POST /api/reset-password
-48 canonical cases • dry-run results until official student ID is supplied</x:v>
+48 canonical cases • official Newman result • X-Student-Id 23127373</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -1492,10 +1522,10 @@
         <x:v>Manual_Review</x:v>
       </x:c>
       <x:c r="L4" s="14" t="str">
-        <x:v>Dry_Result</x:v>
+        <x:v>Official_Result</x:v>
       </x:c>
       <x:c r="M4" s="14" t="str">
-        <x:v>Dry_Failures</x:v>
+        <x:v>Official_Failures</x:v>
       </x:c>
       <x:c r="N4" s="14" t="str">
         <x:v>Human_Verified</x:v>
@@ -3529,7 +3559,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fe22ed0470b4d21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ce2dee90a4041ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3558,7 +3588,7 @@
     <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="4" t="str">
         <x:v>POST /api/apply-coupon
-49 canonical cases • dry-run results until official student ID is supplied</x:v>
+49 canonical cases • official Newman result • X-Student-Id 23127373</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -3627,10 +3657,10 @@
         <x:v>Manual_Review</x:v>
       </x:c>
       <x:c r="L4" s="14" t="str">
-        <x:v>Dry_Result</x:v>
+        <x:v>Official_Result</x:v>
       </x:c>
       <x:c r="M4" s="14" t="str">
-        <x:v>Dry_Failures</x:v>
+        <x:v>Official_Failures</x:v>
       </x:c>
       <x:c r="N4" s="14" t="str">
         <x:v>Human_Verified</x:v>
@@ -5699,7 +5729,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01ab352bdeb94200"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R923abda0bda445c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5728,7 +5758,7 @@
     <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="4" t="str">
         <x:v>POST /api/admin/import-products
-61 canonical cases • dry-run results until official student ID is supplied</x:v>
+61 canonical cases • official Newman result • X-Student-Id 23127373</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -5797,10 +5827,10 @@
         <x:v>Manual_Review</x:v>
       </x:c>
       <x:c r="L4" s="14" t="str">
-        <x:v>Dry_Result</x:v>
+        <x:v>Official_Result</x:v>
       </x:c>
       <x:c r="M4" s="14" t="str">
-        <x:v>Dry_Failures</x:v>
+        <x:v>Official_Failures</x:v>
       </x:c>
       <x:c r="N4" s="14" t="str">
         <x:v>Human_Verified</x:v>
@@ -8375,7 +8405,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3f0dc6a358e4c7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bc593a037454a77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8657,7 +8687,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc82d90f169d4b61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R669890bec940483f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8672,18 +8702,20 @@
     <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
       <x:c r="A1" s="4" t="str">
         <x:v>Genuine Defect Summary
-URLs/screenshots remain human-review gates until publication is approved</x:v>
+Ten issue records with traceable screenshot and official Newman evidence</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
       <x:c r="D1" s="4"/>
       <x:c r="E1" s="4"/>
       <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="4"/>
@@ -8692,6 +8724,7 @@
       <x:c r="D2" s="4"/>
       <x:c r="E2" s="4"/>
       <x:c r="F2" s="4"/>
+      <x:c r="G2" s="4"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="13" t="str">
@@ -8709,8 +8742,11 @@
       <x:c r="E4" s="14" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="F4" s="15" t="str">
+      <x:c r="F4" s="14" t="str">
         <x:v>GitHub_Status</x:v>
+      </x:c>
+      <x:c r="G4" s="15" t="str">
+        <x:v>Issue_URL</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -8730,8 +8766,9 @@
         <x:v>R-H-05; source review</x:v>
       </x:c>
       <x:c r="F5" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G5" s="16" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16" t="str">
@@ -8750,8 +8787,9 @@
         <x:v>R-AI-05..10,35..38</x:v>
       </x:c>
       <x:c r="F6" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="str">
@@ -8770,8 +8808,9 @@
         <x:v>R-AI-15; source review</x:v>
       </x:c>
       <x:c r="F7" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="16" t="str">
@@ -8790,8 +8829,9 @@
         <x:v>C-AI-02..09</x:v>
       </x:c>
       <x:c r="F8" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="str">
@@ -8810,8 +8850,9 @@
         <x:v>C-AI-01,19,34</x:v>
       </x:c>
       <x:c r="F9" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="16" t="str">
@@ -8830,8 +8871,9 @@
         <x:v>C-AI-18,21,22</x:v>
       </x:c>
       <x:c r="F10" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="16" t="str">
@@ -8850,8 +8892,9 @@
         <x:v>I-AI-02,56</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="16" t="str">
@@ -8870,8 +8913,9 @@
         <x:v>I-AI-21..33</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G12" s="16" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="16" t="str">
@@ -8890,8 +8934,9 @@
         <x:v>I-AI-40..42,51</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G13" s="16" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="16" t="str">
@@ -8910,20 +8955,21 @@
         <x:v>R/C/I malformed rows</x:v>
       </x:c>
       <x:c r="F14" s="16" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="G14" s="16" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:F2"/>
+    <x:mergeCell ref="A1:G2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B5:B14">
-    <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="Critical"/>
-    <x:cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="High"/>
+    <x:cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="Critical"/>
+    <x:cfRule type="containsText" dxfId="20" priority="2" operator="containsText" text="High"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6486d7fb04e43be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3f8591d977942b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8984,7 +9030,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
         <x:v>Student</x:v>
@@ -9012,7 +9058,7 @@
         <x:v>MR-03</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>Run official Newman command and capture real console header</x:v>
+        <x:v>Capture/recreate the real official Newman console header screenshot</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
         <x:v>BLOCKING</x:v>
@@ -9046,7 +9092,7 @@
         <x:v>MR-05</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Publish issues with real screenshots</x:v>
+        <x:v>Publish issues with real screenshot links</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
         <x:v>BLOCKING</x:v>
@@ -9069,7 +9115,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D10" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
         <x:v>Student</x:v>
@@ -9148,8 +9194,8 @@
     <x:mergeCell ref="A1:E2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="D5:D14">
-    <x:cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="NO"/>
-    <x:cfRule type="containsText" dxfId="21" priority="2" operator="containsText" text="YES"/>
+    <x:cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="NO"/>
+    <x:cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="YES"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="D5:D14">
@@ -9158,7 +9204,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4c8aeba485348b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81d4a83875a44411"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: publish ten verified defect issues
</commit_message>
<xml_diff>
--- a/outputs/hw06/HW06_Test_Cases.xlsx
+++ b/outputs/hw06/HW06_Test_Cases.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R31dc64276ff34331"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="Rd508a98d75b042f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="Rd9aab81921e84b0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="R65c0221703344d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="Rb379b6e4ba3248d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="R8c28afe74a5a4bf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="R5a05c2aa6fcf45a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdda47d8b9aa34e34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="Re5572fcfede4498a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="R0ebb007507614968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="R1ecfd773e7ab4910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="R840d4bb4c6e446b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="R1b7d66ab1098436f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="Rbb896621abf64a58"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -661,7 +661,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1cc720a8b94c496b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R507cf1bb5d934494"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1307,7 +1307,7 @@
         <x:v>GitHub Issues</x:v>
       </x:c>
       <x:c r="E15" s="37" t="n">
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F15" s="37" t="str">
         <x:v>10 expected</x:v>
@@ -1321,7 +1321,7 @@
         <x:v>Ten GitHub Issues</x:v>
       </x:c>
       <x:c r="B16" s="42" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="C16" s="37"/>
       <x:c r="D16" s="37" t="str">
@@ -1425,7 +1425,7 @@
     <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="YES"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64ced6bb13b74d5f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eace2ece22e48ae"/>
 </x:worksheet>
 </file>
 
@@ -3559,7 +3559,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ce2dee90a4041ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R943219f9eb7c4b53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5729,7 +5729,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R923abda0bda445c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b4bbd78eb6946a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8405,7 +8405,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bc593a037454a77"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3e88fbe27294f5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8687,7 +8687,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R669890bec940483f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb56f9d980f154213"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8766,9 +8766,11 @@
         <x:v>R-H-05; source review</x:v>
       </x:c>
       <x:c r="F5" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G5" s="16" t="str"/>
+        <x:v>#1</x:v>
+      </x:c>
+      <x:c r="G5" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/1</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16" t="str">
@@ -8787,9 +8789,11 @@
         <x:v>R-AI-05..10,35..38</x:v>
       </x:c>
       <x:c r="F6" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G6" s="16" t="str"/>
+        <x:v>#2</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/2</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="str">
@@ -8808,9 +8812,11 @@
         <x:v>R-AI-15; source review</x:v>
       </x:c>
       <x:c r="F7" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G7" s="16" t="str"/>
+        <x:v>#3</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/3</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="16" t="str">
@@ -8829,9 +8835,11 @@
         <x:v>C-AI-02..09</x:v>
       </x:c>
       <x:c r="F8" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G8" s="16" t="str"/>
+        <x:v>#4</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/4</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="str">
@@ -8850,9 +8858,11 @@
         <x:v>C-AI-01,19,34</x:v>
       </x:c>
       <x:c r="F9" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G9" s="16" t="str"/>
+        <x:v>#5</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/5</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="16" t="str">
@@ -8871,9 +8881,11 @@
         <x:v>C-AI-18,21,22</x:v>
       </x:c>
       <x:c r="F10" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G10" s="16" t="str"/>
+        <x:v>#6</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/6</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="16" t="str">
@@ -8892,9 +8904,11 @@
         <x:v>I-AI-02,56</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G11" s="16" t="str"/>
+        <x:v>#7</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/7</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="16" t="str">
@@ -8913,9 +8927,11 @@
         <x:v>I-AI-21..33</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G12" s="16" t="str"/>
+        <x:v>#8</x:v>
+      </x:c>
+      <x:c r="G12" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/8</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="16" t="str">
@@ -8934,9 +8950,11 @@
         <x:v>I-AI-40..42,51</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G13" s="16" t="str"/>
+        <x:v>#9</x:v>
+      </x:c>
+      <x:c r="G13" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/9</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="16" t="str">
@@ -8955,9 +8973,11 @@
         <x:v>R/C/I malformed rows</x:v>
       </x:c>
       <x:c r="F14" s="16" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G14" s="16" t="str"/>
+        <x:v>#10</x:v>
+      </x:c>
+      <x:c r="G14" s="16" t="str">
+        <x:v>https://github.com/z3nz3nn/HW06-software-testing/issues/10</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -8969,7 +8989,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3f8591d977942b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab2b0d18c75f44b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9098,7 +9118,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
         <x:v>Student</x:v>
@@ -9204,7 +9224,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81d4a83875a44411"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31eed5b7cfa24efe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: synchronize submission evidence and readiness
</commit_message>
<xml_diff>
--- a/outputs/hw06/HW06_Test_Cases.xlsx
+++ b/outputs/hw06/HW06_Test_Cases.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdda47d8b9aa34e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="Re5572fcfede4498a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="R0ebb007507614968"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="R1ecfd773e7ab4910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="R840d4bb4c6e446b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="R1b7d66ab1098436f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="Rbb896621abf64a58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra3cdbd20c73e429f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="R7c72bef426a449b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="R0c5e7ea5c55b4d85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="R835c853bda414d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="Rd9dfbbddb73f44fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="R5f2b07348f104974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="Rf6cdb181b78a4801"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -661,7 +661,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R507cf1bb5d934494"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc6db3f20854b476e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -769,7 +769,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ManualReviewTable" displayName="ManualReviewTable" ref="A4:E14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ManualReviewTable" displayName="ManualReviewTable" ref="A4:E16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Gate_ID"/>
     <x:tableColumn id="2" name="Required action"/>
@@ -1425,7 +1425,7 @@
     <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="YES"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eace2ece22e48ae"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R188c7ab6bf554631"/>
 </x:worksheet>
 </file>
 
@@ -3559,7 +3559,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R943219f9eb7c4b53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b32a5f8603e4d7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5729,7 +5729,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b4bbd78eb6946a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94b4ae4d01254d5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8405,7 +8405,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3e88fbe27294f5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9cedf590f0548d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8687,7 +8687,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb56f9d980f154213"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84811daccfd7460c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8989,7 +8989,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab2b0d18c75f44b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R915253cc69404b70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9095,7 +9095,7 @@
         <x:v>MR-04</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>Approve/publicize GitHub repository</x:v>
+        <x:v>Personally spot-check the three latest Newman HTML reports</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str">
         <x:v>BLOCKING</x:v>
@@ -9112,13 +9112,13 @@
         <x:v>MR-05</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Publish issues with real screenshot links</x:v>
+        <x:v>Approve/publicize GitHub repository</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
-        <x:v>YES</x:v>
+        <x:v>NO</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
         <x:v>Student</x:v>
@@ -9129,7 +9129,7 @@
         <x:v>MR-06</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>Verify both GitHub Actions demonstration runs</x:v>
+        <x:v>Publish issues with real screenshot links</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
         <x:v>BLOCKING</x:v>
@@ -9146,13 +9146,13 @@
         <x:v>MR-07</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>Draw and export the Agent Skill diagram personally</x:v>
+        <x:v>Verify both GitHub Actions demonstration runs</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D11" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str">
         <x:v>Student</x:v>
@@ -9163,7 +9163,7 @@
         <x:v>MR-08</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
-        <x:v>Record/upload video and add URL</x:v>
+        <x:v>Draw and export the Agent Skill diagram personally</x:v>
       </x:c>
       <x:c r="C12" s="16" t="str">
         <x:v>BLOCKING</x:v>
@@ -9180,7 +9180,7 @@
         <x:v>MR-09</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
-        <x:v>Select self-assessed grade and filename</x:v>
+        <x:v>Personally confirm the AI Audit against Gemini</x:v>
       </x:c>
       <x:c r="C13" s="16" t="str">
         <x:v>BLOCKING</x:v>
@@ -9197,7 +9197,7 @@
         <x:v>MR-10</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
-        <x:v>Inspect ZIP and submit on Moodle</x:v>
+        <x:v>Record/upload video and add URL</x:v>
       </x:c>
       <x:c r="C14" s="16" t="str">
         <x:v>BLOCKING</x:v>
@@ -9206,6 +9206,40 @@
         <x:v>NO</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
+        <x:v>Student</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="16" t="str">
+        <x:v>MR-11</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="str">
+        <x:v>Select self-assessed grade and filename</x:v>
+      </x:c>
+      <x:c r="C15" s="16" t="str">
+        <x:v>BLOCKING</x:v>
+      </x:c>
+      <x:c r="D15" s="16" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="E15" s="16" t="str">
+        <x:v>Student</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="16" t="str">
+        <x:v>MR-12</x:v>
+      </x:c>
+      <x:c r="B16" s="16" t="str">
+        <x:v>Inspect ZIP and submit on Moodle</x:v>
+      </x:c>
+      <x:c r="C16" s="16" t="str">
+        <x:v>BLOCKING</x:v>
+      </x:c>
+      <x:c r="D16" s="16" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="E16" s="16" t="str">
         <x:v>Student</x:v>
       </x:c>
     </x:row>
@@ -9213,18 +9247,18 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:E2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D5:D14">
+  <x:conditionalFormatting sqref="D5:D16">
     <x:cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="NO"/>
     <x:cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="YES"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="D5:D14">
+    <x:dataValidation type="list" sqref="D5:D16">
       <x:formula1>"NO,YES"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31eed5b7cfa24efe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra09823651ff54d2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: prepare submission package and Mermaid diagram
</commit_message>
<xml_diff>
--- a/outputs/hw06/HW06_Test_Cases.xlsx
+++ b/outputs/hw06/HW06_Test_Cases.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra3cdbd20c73e429f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="R7c72bef426a449b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="R0c5e7ea5c55b4d85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="R835c853bda414d34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="Rd9dfbbddb73f44fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="R5f2b07348f104974"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="Rf6cdb181b78a4801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Raa03ca77583d49cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="R84bd94da38654ae6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="Re075a29d1c414f9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="Ra3cf1eb424c04696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="R3db39c27ee844e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="Rabbfb2ba56a64fc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="R9e4efa68453f4ccd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -239,7 +239,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="23">
+  <x:dxfs count="25">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -435,6 +435,28 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4E5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF067647"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFEAF8F0"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF067647"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFEAF8F0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -661,7 +683,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc6db3f20854b476e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raa1753e43e6c4fca"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -985,6 +1007,9 @@
     <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="19" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -1354,10 +1379,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="37" t="str">
-        <x:v>Video + final ZIP</x:v>
+        <x:v>Video decision</x:v>
       </x:c>
       <x:c r="B18" s="42" t="str">
-        <x:v>NO</x:v>
+        <x:v>DECLINED (OPTIONAL)</x:v>
       </x:c>
       <x:c r="C18" s="37"/>
       <x:c r="D18" s="37"/>
@@ -1367,7 +1392,35 @@
       <x:c r="H18" s="37"/>
       <x:c r="I18" s="37"/>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="37" t="str">
+        <x:v>Self-assessed grade</x:v>
+      </x:c>
+      <x:c r="B19" s="42" t="str">
+        <x:v>100/100</x:v>
+      </x:c>
+      <x:c r="C19" s="37"/>
+      <x:c r="D19" s="37"/>
+      <x:c r="E19" s="37"/>
+      <x:c r="F19" s="37"/>
+      <x:c r="G19" s="37"/>
+      <x:c r="H19" s="37"/>
+      <x:c r="I19" s="37"/>
+    </x:row>
     <x:row r="20">
+      <x:c r="A20" s="37" t="str">
+        <x:v>Final ZIP inspected</x:v>
+      </x:c>
+      <x:c r="B20" s="42" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="C20" s="37"/>
+      <x:c r="D20" s="37"/>
+      <x:c r="E20" s="37"/>
+      <x:c r="F20" s="37"/>
+      <x:c r="G20" s="37"/>
+      <x:c r="H20" s="37"/>
+      <x:c r="I20" s="37"/>
       <x:c r="K20" t="str">
         <x:v>API</x:v>
       </x:c>
@@ -1421,11 +1474,13 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:I2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="B12:B18">
+  <x:conditionalFormatting sqref="B12:B20">
     <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="YES"/>
+    <x:cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="OPTIONAL"/>
+    <x:cfRule type="containsText" dxfId="20" priority="3" operator="containsText" text="/100"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R188c7ab6bf554631"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3212bf290e6240c1"/>
 </x:worksheet>
 </file>
 
@@ -3559,7 +3614,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b32a5f8603e4d7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf278933515734533"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5729,7 +5784,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94b4ae4d01254d5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0960ac75023949cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8405,7 +8460,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9cedf590f0548d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a2d259f3fc439e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8687,7 +8742,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84811daccfd7460c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8e67f7c060c4ee0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8984,12 +9039,12 @@
     <x:mergeCell ref="A1:G2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B5:B14">
-    <x:cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="Critical"/>
-    <x:cfRule type="containsText" dxfId="20" priority="2" operator="containsText" text="High"/>
+    <x:cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="Critical"/>
+    <x:cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="High"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R915253cc69404b70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7319e86383fd424a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9197,13 +9252,13 @@
         <x:v>MR-10</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
-        <x:v>Record/upload video and add URL</x:v>
+        <x:v>Optional video explicitly declined</x:v>
       </x:c>
       <x:c r="C14" s="16" t="str">
-        <x:v>BLOCKING</x:v>
+        <x:v>OPTIONAL</x:v>
       </x:c>
       <x:c r="D14" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
         <x:v>Student</x:v>
@@ -9220,7 +9275,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D15" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
         <x:v>Student</x:v>
@@ -9248,8 +9303,8 @@
     <x:mergeCell ref="A1:E2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="D5:D16">
-    <x:cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="NO"/>
-    <x:cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="YES"/>
+    <x:cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="NO"/>
+    <x:cfRule type="containsText" dxfId="24" priority="2" operator="containsText" text="YES"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="D5:D16">
@@ -9258,7 +9313,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra09823651ff54d2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47ce4670b2b54e01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record completed evidence review
</commit_message>
<xml_diff>
--- a/outputs/hw06/HW06_Test_Cases.xlsx
+++ b/outputs/hw06/HW06_Test_Cases.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Raa03ca77583d49cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="R84bd94da38654ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="Re075a29d1c414f9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="Ra3cf1eb424c04696"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="R3db39c27ee844e3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="Rabbfb2ba56a64fc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="R9e4efa68453f4ccd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra2ff1d76981a4844"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="R340518ee2fba4600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="R44810980d808440b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="Rc7f8c0b94bff4249"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="R8c6034ad32964dc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="R8fa87e8b6f35443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="Re128b7480cb94576"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -239,7 +239,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="25">
+  <x:dxfs count="28">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -303,6 +303,17 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4E5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF067647"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFEAF8F0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -375,6 +386,17 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF067647"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFEAF8F0"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
@@ -435,6 +457,17 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4E5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF067647"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFEAF8F0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -683,7 +716,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raa1753e43e6c4fca"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R29e19f29abb64de4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1304,7 +1337,7 @@
         <x:v>Rows personally reviewed</x:v>
       </x:c>
       <x:c r="B14" s="42" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="C14" s="37"/>
       <x:c r="D14" s="37" t="str">
@@ -1325,7 +1358,7 @@
         <x:v>Self-drawn diagram</x:v>
       </x:c>
       <x:c r="B15" s="42" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="C15" s="37"/>
       <x:c r="D15" s="37" t="str">
@@ -1475,12 +1508,12 @@
     <x:mergeCell ref="A1:I2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B12:B20">
-    <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="YES"/>
-    <x:cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="OPTIONAL"/>
-    <x:cfRule type="containsText" dxfId="20" priority="3" operator="containsText" text="/100"/>
+    <x:cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="YES"/>
+    <x:cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="OPTIONAL"/>
+    <x:cfRule type="containsText" dxfId="23" priority="3" operator="containsText" text="/100"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3212bf290e6240c1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8930911bef34d5d"/>
 </x:worksheet>
 </file>
 
@@ -1626,9 +1659,11 @@
       </x:c>
       <x:c r="M5" s="17" t="str"/>
       <x:c r="N5" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O5" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O5" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="17" t="str">
@@ -1667,9 +1702,11 @@
       </x:c>
       <x:c r="M6" s="17" t="str"/>
       <x:c r="N6" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O6" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O6" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="17" t="str">
@@ -1708,9 +1745,11 @@
       </x:c>
       <x:c r="M7" s="17" t="str"/>
       <x:c r="N7" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O7" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O7" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="17" t="str">
@@ -1749,9 +1788,11 @@
       </x:c>
       <x:c r="M8" s="17" t="str"/>
       <x:c r="N8" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O8" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O8" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="17" t="str">
@@ -1792,9 +1833,11 @@
         <x:v>[R-AI-05] no success response for invalid reset | [R-AI-05] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N9" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O9" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O9" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="17" t="str">
@@ -1835,9 +1878,11 @@
         <x:v>[R-AI-06] no success response for invalid reset | [R-AI-06] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N10" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O10" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O10" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="17" t="str">
@@ -1878,9 +1923,11 @@
         <x:v>[R-AI-07] no success response for invalid reset | [R-AI-07] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N11" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O11" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O11" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="17" t="str">
@@ -1921,9 +1968,11 @@
         <x:v>[R-AI-08] no success response for invalid reset | [R-AI-08] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N12" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O12" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O12" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="17" t="str">
@@ -1964,9 +2013,11 @@
         <x:v>[R-AI-09] no success response for invalid reset | [R-AI-09] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N13" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O13" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O13" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="17" t="str">
@@ -2007,9 +2058,11 @@
         <x:v>[R-AI-10] no success response for invalid reset | [R-AI-10] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N14" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O14" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O14" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="17" t="str">
@@ -2048,9 +2101,11 @@
       </x:c>
       <x:c r="M15" s="17" t="str"/>
       <x:c r="N15" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O15" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O15" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="17" t="str">
@@ -2089,9 +2144,11 @@
       </x:c>
       <x:c r="M16" s="17" t="str"/>
       <x:c r="N16" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O16" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O16" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="17" t="str">
@@ -2130,9 +2187,11 @@
       </x:c>
       <x:c r="M17" s="17" t="str"/>
       <x:c r="N17" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O17" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O17" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="17" t="str">
@@ -2171,9 +2230,11 @@
       </x:c>
       <x:c r="M18" s="17" t="str"/>
       <x:c r="N18" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O18" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O18" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="17" t="str">
@@ -2214,9 +2275,11 @@
       </x:c>
       <x:c r="M19" s="17" t="str"/>
       <x:c r="N19" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O19" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O19" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="17" t="str">
@@ -2255,9 +2318,11 @@
       </x:c>
       <x:c r="M20" s="17" t="str"/>
       <x:c r="N20" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O20" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O20" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="17" t="str">
@@ -2296,9 +2361,11 @@
       </x:c>
       <x:c r="M21" s="17" t="str"/>
       <x:c r="N21" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O21" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O21" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="17" t="str">
@@ -2337,9 +2404,11 @@
       </x:c>
       <x:c r="M22" s="17" t="str"/>
       <x:c r="N22" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O22" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O22" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="17" t="str">
@@ -2378,9 +2447,11 @@
       </x:c>
       <x:c r="M23" s="17" t="str"/>
       <x:c r="N23" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O23" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O23" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="17" t="str">
@@ -2419,9 +2490,11 @@
       </x:c>
       <x:c r="M24" s="17" t="str"/>
       <x:c r="N24" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O24" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O24" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="17" t="str">
@@ -2460,9 +2533,11 @@
       </x:c>
       <x:c r="M25" s="17" t="str"/>
       <x:c r="N25" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O25" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O25" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="17" t="str">
@@ -2501,9 +2576,11 @@
       </x:c>
       <x:c r="M26" s="17" t="str"/>
       <x:c r="N26" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O26" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O26" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="17" t="str">
@@ -2544,9 +2621,11 @@
       </x:c>
       <x:c r="M27" s="17" t="str"/>
       <x:c r="N27" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O27" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O27" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="17" t="str">
@@ -2585,9 +2664,11 @@
       </x:c>
       <x:c r="M28" s="17" t="str"/>
       <x:c r="N28" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O28" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O28" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="17" t="str">
@@ -2626,9 +2707,11 @@
       </x:c>
       <x:c r="M29" s="17" t="str"/>
       <x:c r="N29" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O29" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O29" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="17" t="str">
@@ -2667,9 +2750,11 @@
       </x:c>
       <x:c r="M30" s="17" t="str"/>
       <x:c r="N30" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O30" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O30" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="17" t="str">
@@ -2708,9 +2793,11 @@
       </x:c>
       <x:c r="M31" s="17" t="str"/>
       <x:c r="N31" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O31" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O31" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="17" t="str">
@@ -2749,9 +2836,11 @@
       </x:c>
       <x:c r="M32" s="17" t="str"/>
       <x:c r="N32" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O32" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O32" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="17" t="str">
@@ -2790,9 +2879,11 @@
       </x:c>
       <x:c r="M33" s="17" t="str"/>
       <x:c r="N33" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O33" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O33" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="17" t="str">
@@ -2831,9 +2922,11 @@
       </x:c>
       <x:c r="M34" s="17" t="str"/>
       <x:c r="N34" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O34" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O34" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="17" t="str">
@@ -2872,9 +2965,11 @@
       </x:c>
       <x:c r="M35" s="17" t="str"/>
       <x:c r="N35" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O35" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O35" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="17" t="str">
@@ -2913,9 +3008,11 @@
       </x:c>
       <x:c r="M36" s="17" t="str"/>
       <x:c r="N36" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O36" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O36" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="17" t="str">
@@ -2954,9 +3051,11 @@
       </x:c>
       <x:c r="M37" s="17" t="str"/>
       <x:c r="N37" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O37" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O37" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="17" t="str">
@@ -2995,9 +3094,11 @@
       </x:c>
       <x:c r="M38" s="17" t="str"/>
       <x:c r="N38" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O38" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O38" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="17" t="str">
@@ -3038,9 +3139,11 @@
         <x:v>[R-AI-35] no success response for invalid reset | [R-AI-35] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N39" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O39" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O39" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="17" t="str">
@@ -3081,9 +3184,11 @@
         <x:v>[R-AI-36] no success response for invalid reset | [R-AI-36] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N40" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O40" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O40" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="17" t="str">
@@ -3124,9 +3229,11 @@
         <x:v>[R-AI-37] no success response for invalid reset | [R-AI-37] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N41" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O41" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O41" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="17" t="str">
@@ -3167,9 +3274,11 @@
         <x:v>[R-AI-38] no success response for invalid reset | [R-AI-38] password state matches the normative oracle</x:v>
       </x:c>
       <x:c r="N42" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O42" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O42" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="17" t="str">
@@ -3208,9 +3317,11 @@
       </x:c>
       <x:c r="M43" s="17" t="str"/>
       <x:c r="N43" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O43" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O43" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="17" t="str">
@@ -3251,9 +3362,11 @@
         <x:v>[R-AI-40] response has no stack/database leak</x:v>
       </x:c>
       <x:c r="N44" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O44" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O44" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="17" t="str">
@@ -3292,9 +3405,11 @@
       </x:c>
       <x:c r="M45" s="17" t="str"/>
       <x:c r="N45" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O45" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O45" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="17" t="str">
@@ -3333,9 +3448,11 @@
       </x:c>
       <x:c r="M46" s="17" t="str"/>
       <x:c r="N46" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O46" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O46" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="17" t="str">
@@ -3376,9 +3493,11 @@
         <x:v>[R-H-01] response has no stack/database leak</x:v>
       </x:c>
       <x:c r="N47" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O47" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O47" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="17" t="str">
@@ -3419,9 +3538,11 @@
       </x:c>
       <x:c r="M48" s="17" t="str"/>
       <x:c r="N48" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O48" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O48" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="17" t="str">
@@ -3460,9 +3581,11 @@
       </x:c>
       <x:c r="M49" s="17" t="str"/>
       <x:c r="N49" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O49" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O49" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
       <x:c r="A50" s="17" t="str">
@@ -3501,9 +3624,11 @@
       </x:c>
       <x:c r="M50" s="17" t="str"/>
       <x:c r="N50" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O50" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O50" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
       <x:c r="A51" s="17" t="str">
@@ -3544,9 +3669,11 @@
         <x:v>Login response does not disclose stored secrets</x:v>
       </x:c>
       <x:c r="N51" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O51" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O51" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
       <x:c r="A52" s="17" t="str">
@@ -3587,9 +3714,11 @@
       </x:c>
       <x:c r="M52" s="17" t="str"/>
       <x:c r="N52" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O52" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O52" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3606,6 +3735,7 @@
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="N5:N52">
     <x:cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="NO"/>
+    <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="YES"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="N5:N52">
@@ -3614,7 +3744,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf278933515734533"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R563776ffe5e14c1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3763,9 +3893,11 @@
         <x:v>discount_amount follows formula | final_amount follows formula</x:v>
       </x:c>
       <x:c r="N5" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O5" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O5" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="17" t="str">
@@ -3806,9 +3938,11 @@
         <x:v>[C-AI-02] coupon is not applied</x:v>
       </x:c>
       <x:c r="N6" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O6" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O6" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="17" t="str">
@@ -3849,9 +3983,11 @@
         <x:v>[C-AI-03] coupon is not applied</x:v>
       </x:c>
       <x:c r="N7" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O7" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O7" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="17" t="str">
@@ -3892,9 +4028,11 @@
         <x:v>[C-AI-04] coupon is not applied</x:v>
       </x:c>
       <x:c r="N8" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O8" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O8" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="17" t="str">
@@ -3935,9 +4073,11 @@
         <x:v>[C-AI-05] coupon is not applied</x:v>
       </x:c>
       <x:c r="N9" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O9" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O9" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="17" t="str">
@@ -3978,9 +4118,11 @@
         <x:v>[C-AI-06] coupon is not applied</x:v>
       </x:c>
       <x:c r="N10" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O10" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O10" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="17" t="str">
@@ -4019,9 +4161,11 @@
       </x:c>
       <x:c r="M11" s="17" t="str"/>
       <x:c r="N11" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O11" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O11" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="17" t="str">
@@ -4060,9 +4204,11 @@
       </x:c>
       <x:c r="M12" s="17" t="str"/>
       <x:c r="N12" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O12" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O12" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="17" t="str">
@@ -4103,9 +4249,11 @@
         <x:v>[C-AI-09] coupon is not applied</x:v>
       </x:c>
       <x:c r="N13" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O13" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O13" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="17" t="str">
@@ -4144,9 +4292,11 @@
       </x:c>
       <x:c r="M14" s="17" t="str"/>
       <x:c r="N14" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O14" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O14" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="17" t="str">
@@ -4185,9 +4335,11 @@
       </x:c>
       <x:c r="M15" s="17" t="str"/>
       <x:c r="N15" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O15" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O15" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="17" t="str">
@@ -4226,9 +4378,11 @@
       </x:c>
       <x:c r="M16" s="17" t="str"/>
       <x:c r="N16" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O16" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O16" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="17" t="str">
@@ -4267,9 +4421,11 @@
       </x:c>
       <x:c r="M17" s="17" t="str"/>
       <x:c r="N17" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O17" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O17" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="17" t="str">
@@ -4308,9 +4464,11 @@
       </x:c>
       <x:c r="M18" s="17" t="str"/>
       <x:c r="N18" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O18" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O18" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="17" t="str">
@@ -4349,9 +4507,11 @@
       </x:c>
       <x:c r="M19" s="17" t="str"/>
       <x:c r="N19" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O19" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O19" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="17" t="str">
@@ -4390,9 +4550,11 @@
       </x:c>
       <x:c r="M20" s="17" t="str"/>
       <x:c r="N20" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O20" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O20" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="17" t="str">
@@ -4431,9 +4593,11 @@
       </x:c>
       <x:c r="M21" s="17" t="str"/>
       <x:c r="N21" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O21" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O21" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="17" t="str">
@@ -4474,9 +4638,11 @@
         <x:v>[C-AI-18] coupon applies | Required numeric success fields exist | discount_amount follows formula | final_amount follows formula | Core formula invariant</x:v>
       </x:c>
       <x:c r="N22" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O22" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O22" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="17" t="str">
@@ -4517,9 +4683,11 @@
         <x:v>discount_amount follows formula | final_amount follows formula</x:v>
       </x:c>
       <x:c r="N23" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O23" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O23" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="17" t="str">
@@ -4558,9 +4726,11 @@
       </x:c>
       <x:c r="M24" s="17" t="str"/>
       <x:c r="N24" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O24" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O24" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="17" t="str">
@@ -4601,9 +4771,11 @@
         <x:v>[C-AI-21] coupon applies | Required numeric success fields exist | discount_amount follows formula | final_amount follows formula | Core formula invariant</x:v>
       </x:c>
       <x:c r="N25" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O25" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O25" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="17" t="str">
@@ -4644,9 +4816,11 @@
         <x:v>[C-AI-22] coupon applies | Required numeric success fields exist | discount_amount follows formula | final_amount follows formula | Core formula invariant</x:v>
       </x:c>
       <x:c r="N26" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O26" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O26" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="17" t="str">
@@ -4685,9 +4859,11 @@
       </x:c>
       <x:c r="M27" s="17" t="str"/>
       <x:c r="N27" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O27" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O27" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="17" t="str">
@@ -4726,9 +4902,11 @@
       </x:c>
       <x:c r="M28" s="17" t="str"/>
       <x:c r="N28" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O28" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O28" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="17" t="str">
@@ -4767,9 +4945,11 @@
       </x:c>
       <x:c r="M29" s="17" t="str"/>
       <x:c r="N29" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O29" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O29" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="17" t="str">
@@ -4808,9 +4988,11 @@
       </x:c>
       <x:c r="M30" s="17" t="str"/>
       <x:c r="N30" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O30" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O30" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="17" t="str">
@@ -4849,9 +5031,11 @@
       </x:c>
       <x:c r="M31" s="17" t="str"/>
       <x:c r="N31" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O31" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O31" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="17" t="str">
@@ -4890,9 +5074,11 @@
       </x:c>
       <x:c r="M32" s="17" t="str"/>
       <x:c r="N32" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O32" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O32" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="17" t="str">
@@ -4931,9 +5117,11 @@
       </x:c>
       <x:c r="M33" s="17" t="str"/>
       <x:c r="N33" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O33" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O33" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="17" t="str">
@@ -4972,9 +5160,11 @@
       </x:c>
       <x:c r="M34" s="17" t="str"/>
       <x:c r="N34" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O34" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O34" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="17" t="str">
@@ -5013,9 +5203,11 @@
       </x:c>
       <x:c r="M35" s="17" t="str"/>
       <x:c r="N35" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O35" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O35" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="17" t="str">
@@ -5054,9 +5246,11 @@
       </x:c>
       <x:c r="M36" s="17" t="str"/>
       <x:c r="N36" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O36" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O36" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="17" t="str">
@@ -5097,9 +5291,11 @@
         <x:v>discount_amount follows formula | final_amount follows formula</x:v>
       </x:c>
       <x:c r="N37" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O37" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O37" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="17" t="str">
@@ -5138,9 +5334,11 @@
       </x:c>
       <x:c r="M38" s="17" t="str"/>
       <x:c r="N38" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O38" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O38" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="17" t="str">
@@ -5179,9 +5377,11 @@
       </x:c>
       <x:c r="M39" s="17" t="str"/>
       <x:c r="N39" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O39" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O39" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="17" t="str">
@@ -5220,9 +5420,11 @@
       </x:c>
       <x:c r="M40" s="17" t="str"/>
       <x:c r="N40" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O40" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O40" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="17" t="str">
@@ -5261,9 +5463,11 @@
       </x:c>
       <x:c r="M41" s="17" t="str"/>
       <x:c r="N41" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O41" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O41" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="17" t="str">
@@ -5302,9 +5506,11 @@
       </x:c>
       <x:c r="M42" s="17" t="str"/>
       <x:c r="N42" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O42" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O42" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="17" t="str">
@@ -5345,9 +5551,11 @@
         <x:v>[C-AI-40] response has no stack/database leak</x:v>
       </x:c>
       <x:c r="N43" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O43" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O43" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="17" t="str">
@@ -5386,9 +5594,11 @@
       </x:c>
       <x:c r="M44" s="17" t="str"/>
       <x:c r="N44" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O44" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O44" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="17" t="str">
@@ -5427,9 +5637,11 @@
       </x:c>
       <x:c r="M45" s="17" t="str"/>
       <x:c r="N45" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O45" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O45" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="17" t="str">
@@ -5468,9 +5680,11 @@
       </x:c>
       <x:c r="M46" s="17" t="str"/>
       <x:c r="N46" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O46" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O46" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="17" t="str">
@@ -5511,9 +5725,11 @@
       </x:c>
       <x:c r="M47" s="17" t="str"/>
       <x:c r="N47" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O47" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O47" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="17" t="str">
@@ -5552,9 +5768,11 @@
       </x:c>
       <x:c r="M48" s="17" t="str"/>
       <x:c r="N48" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O48" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O48" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="17" t="str">
@@ -5593,9 +5811,11 @@
       </x:c>
       <x:c r="M49" s="17" t="str"/>
       <x:c r="N49" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O49" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O49" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
       <x:c r="A50" s="17" t="str">
@@ -5634,9 +5854,11 @@
       </x:c>
       <x:c r="M50" s="17" t="str"/>
       <x:c r="N50" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O50" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O50" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
       <x:c r="A51" s="17" t="str">
@@ -5675,9 +5897,11 @@
       </x:c>
       <x:c r="M51" s="17" t="str"/>
       <x:c r="N51" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O51" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O51" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
       <x:c r="A52" s="17" t="str">
@@ -5716,9 +5940,11 @@
       </x:c>
       <x:c r="M52" s="17" t="str"/>
       <x:c r="N52" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O52" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O52" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
       <x:c r="A53" s="17" t="str">
@@ -5757,25 +5983,28 @@
       </x:c>
       <x:c r="M53" s="17" t="str"/>
       <x:c r="N53" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O53" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O53" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="D5:D53">
-    <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="INVALID"/>
-    <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="INCOMPLETE"/>
-    <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="STUDENT_ADDED"/>
+    <x:cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="INVALID"/>
+    <x:cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="INCOMPLETE"/>
+    <x:cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="STUDENT_ADDED"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="L5:L53">
-    <x:cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="PASS"/>
-    <x:cfRule type="containsText" dxfId="10" priority="5" operator="containsText" text="FAIL"/>
+    <x:cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="PASS"/>
+    <x:cfRule type="containsText" dxfId="11" priority="5" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="N5:N53">
-    <x:cfRule type="containsText" dxfId="11" priority="6" operator="containsText" text="NO"/>
+    <x:cfRule type="containsText" dxfId="12" priority="6" operator="containsText" text="NO"/>
+    <x:cfRule type="containsText" dxfId="13" priority="7" operator="containsText" text="YES"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="N5:N53">
@@ -5784,7 +6013,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0960ac75023949cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43aab7efe078463a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5931,9 +6160,11 @@
       </x:c>
       <x:c r="M5" s="17" t="str"/>
       <x:c r="N5" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O5" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O5" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="17" t="str">
@@ -5974,9 +6205,11 @@
         <x:v>Authorization gate rejects request | [I-AI-02] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N6" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O6" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O6" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="17" t="str">
@@ -6015,9 +6248,11 @@
       </x:c>
       <x:c r="M7" s="17" t="str"/>
       <x:c r="N7" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O7" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O7" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="17" t="str">
@@ -6056,9 +6291,11 @@
       </x:c>
       <x:c r="M8" s="17" t="str"/>
       <x:c r="N8" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O8" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O8" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="17" t="str">
@@ -6097,9 +6334,11 @@
       </x:c>
       <x:c r="M9" s="17" t="str"/>
       <x:c r="N9" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O9" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O9" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="17" t="str">
@@ -6138,9 +6377,11 @@
       </x:c>
       <x:c r="M10" s="17" t="str"/>
       <x:c r="N10" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O10" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O10" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="17" t="str">
@@ -6179,9 +6420,11 @@
       </x:c>
       <x:c r="M11" s="17" t="str"/>
       <x:c r="N11" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O11" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O11" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="17" t="str">
@@ -6220,9 +6463,11 @@
       </x:c>
       <x:c r="M12" s="17" t="str"/>
       <x:c r="N12" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O12" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O12" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="17" t="str">
@@ -6261,9 +6506,11 @@
       </x:c>
       <x:c r="M13" s="17" t="str"/>
       <x:c r="N13" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O13" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O13" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="17" t="str">
@@ -6302,9 +6549,11 @@
       </x:c>
       <x:c r="M14" s="17" t="str"/>
       <x:c r="N14" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O14" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O14" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="17" t="str">
@@ -6343,9 +6592,11 @@
       </x:c>
       <x:c r="M15" s="17" t="str"/>
       <x:c r="N15" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O15" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O15" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="17" t="str">
@@ -6384,9 +6635,11 @@
       </x:c>
       <x:c r="M16" s="17" t="str"/>
       <x:c r="N16" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O16" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O16" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="17" t="str">
@@ -6425,9 +6678,11 @@
       </x:c>
       <x:c r="M17" s="17" t="str"/>
       <x:c r="N17" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O17" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O17" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="17" t="str">
@@ -6466,9 +6721,11 @@
       </x:c>
       <x:c r="M18" s="17" t="str"/>
       <x:c r="N18" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O18" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O18" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="17" t="str">
@@ -6507,9 +6764,11 @@
       </x:c>
       <x:c r="M19" s="17" t="str"/>
       <x:c r="N19" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O19" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O19" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="17" t="str">
@@ -6548,9 +6807,11 @@
       </x:c>
       <x:c r="M20" s="17" t="str"/>
       <x:c r="N20" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O20" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O20" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="17" t="str">
@@ -6589,9 +6850,11 @@
       </x:c>
       <x:c r="M21" s="17" t="str"/>
       <x:c r="N21" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O21" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O21" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="17" t="str">
@@ -6630,9 +6893,11 @@
       </x:c>
       <x:c r="M22" s="17" t="str"/>
       <x:c r="N22" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O22" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O22" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="17" t="str">
@@ -6671,9 +6936,11 @@
       </x:c>
       <x:c r="M23" s="17" t="str"/>
       <x:c r="N23" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O23" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O23" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="17" t="str">
@@ -6712,9 +6979,11 @@
       </x:c>
       <x:c r="M24" s="17" t="str"/>
       <x:c r="N24" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O24" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O24" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="17" t="str">
@@ -6755,9 +7024,11 @@
         <x:v>[I-AI-21] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N25" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O25" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O25" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="17" t="str">
@@ -6798,9 +7069,11 @@
         <x:v>[I-AI-22] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N26" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O26" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O26" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="17" t="str">
@@ -6841,9 +7114,11 @@
         <x:v>[I-AI-23] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N27" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O27" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O27" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="17" t="str">
@@ -6884,9 +7159,11 @@
         <x:v>[I-AI-24] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N28" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O28" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O28" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="17" t="str">
@@ -6927,9 +7204,11 @@
         <x:v>[I-AI-25] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N29" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O29" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O29" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="17" t="str">
@@ -6968,9 +7247,11 @@
       </x:c>
       <x:c r="M30" s="17" t="str"/>
       <x:c r="N30" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O30" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O30" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="17" t="str">
@@ -7009,9 +7290,11 @@
       </x:c>
       <x:c r="M31" s="17" t="str"/>
       <x:c r="N31" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O31" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O31" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="17" t="str">
@@ -7050,9 +7333,11 @@
       </x:c>
       <x:c r="M32" s="17" t="str"/>
       <x:c r="N32" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O32" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O32" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="17" t="str">
@@ -7091,9 +7376,11 @@
       </x:c>
       <x:c r="M33" s="17" t="str"/>
       <x:c r="N33" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O33" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O33" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="17" t="str">
@@ -7134,9 +7421,11 @@
         <x:v>[I-AI-30] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N34" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O34" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O34" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="17" t="str">
@@ -7177,9 +7466,11 @@
         <x:v>[I-AI-31] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N35" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O35" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O35" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="17" t="str">
@@ -7220,9 +7511,11 @@
         <x:v>[I-AI-32] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N36" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O36" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O36" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="17" t="str">
@@ -7263,9 +7556,11 @@
         <x:v>[I-AI-33] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N37" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O37" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O37" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="17" t="str">
@@ -7304,9 +7599,11 @@
       </x:c>
       <x:c r="M38" s="17" t="str"/>
       <x:c r="N38" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O38" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O38" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="17" t="str">
@@ -7345,9 +7642,11 @@
       </x:c>
       <x:c r="M39" s="17" t="str"/>
       <x:c r="N39" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O39" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O39" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="17" t="str">
@@ -7386,9 +7685,11 @@
       </x:c>
       <x:c r="M40" s="17" t="str"/>
       <x:c r="N40" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O40" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O40" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="17" t="str">
@@ -7427,9 +7728,11 @@
       </x:c>
       <x:c r="M41" s="17" t="str"/>
       <x:c r="N41" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O41" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O41" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="17" t="str">
@@ -7468,9 +7771,11 @@
       </x:c>
       <x:c r="M42" s="17" t="str"/>
       <x:c r="N42" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O42" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O42" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="17" t="str">
@@ -7509,9 +7814,11 @@
       </x:c>
       <x:c r="M43" s="17" t="str"/>
       <x:c r="N43" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O43" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O43" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="17" t="str">
@@ -7552,9 +7859,11 @@
         <x:v>[I-AI-40] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N44" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O44" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O44" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="17" t="str">
@@ -7595,9 +7904,11 @@
         <x:v>[I-AI-41] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N45" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O45" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O45" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="17" t="str">
@@ -7638,9 +7949,11 @@
         <x:v>[I-AI-42] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N46" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O46" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O46" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="17" t="str">
@@ -7679,9 +7992,11 @@
       </x:c>
       <x:c r="M47" s="17" t="str"/>
       <x:c r="N47" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O47" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O47" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="17" t="str">
@@ -7720,9 +8035,11 @@
       </x:c>
       <x:c r="M48" s="17" t="str"/>
       <x:c r="N48" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O48" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O48" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="17" t="str">
@@ -7763,9 +8080,11 @@
         <x:v>[I-AI-45] response has no stack/database leak</x:v>
       </x:c>
       <x:c r="N49" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O49" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O49" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
       <x:c r="A50" s="17" t="str">
@@ -7804,9 +8123,11 @@
       </x:c>
       <x:c r="M50" s="17" t="str"/>
       <x:c r="N50" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O50" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O50" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
       <x:c r="A51" s="17" t="str">
@@ -7845,9 +8166,11 @@
       </x:c>
       <x:c r="M51" s="17" t="str"/>
       <x:c r="N51" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O51" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O51" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
       <x:c r="A52" s="17" t="str">
@@ -7888,9 +8211,11 @@
       </x:c>
       <x:c r="M52" s="17" t="str"/>
       <x:c r="N52" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O52" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O52" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
       <x:c r="A53" s="17" t="str">
@@ -7929,9 +8254,11 @@
       </x:c>
       <x:c r="M53" s="17" t="str"/>
       <x:c r="N53" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O53" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O53" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
       <x:c r="A54" s="17" t="str">
@@ -7970,9 +8297,11 @@
       </x:c>
       <x:c r="M54" s="17" t="str"/>
       <x:c r="N54" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O54" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O54" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
       <x:c r="A55" s="17" t="str">
@@ -8013,9 +8342,11 @@
         <x:v>[I-AI-51] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N55" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O55" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O55" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
       <x:c r="A56" s="17" t="str">
@@ -8054,9 +8385,11 @@
       </x:c>
       <x:c r="M56" s="17" t="str"/>
       <x:c r="N56" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O56" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O56" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="42" customHeight="1">
       <x:c r="A57" s="17" t="str">
@@ -8095,9 +8428,11 @@
       </x:c>
       <x:c r="M57" s="17" t="str"/>
       <x:c r="N57" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O57" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O57" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
       <x:c r="A58" s="17" t="str">
@@ -8138,9 +8473,11 @@
       </x:c>
       <x:c r="M58" s="17" t="str"/>
       <x:c r="N58" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O58" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O58" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="42" customHeight="1">
       <x:c r="A59" s="17" t="str">
@@ -8181,9 +8518,11 @@
         <x:v>[I-AI-55] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N59" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O59" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O59" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
       <x:c r="A60" s="17" t="str">
@@ -8224,9 +8563,11 @@
         <x:v>Authorization gate rejects request | [I-AI-56] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N60" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O60" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O60" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="42" customHeight="1">
       <x:c r="A61" s="17" t="str">
@@ -8267,9 +8608,11 @@
         <x:v>[I-H-01] response has no stack/database leak | [I-H-01] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N61" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O61" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O61" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="42" customHeight="1">
       <x:c r="A62" s="17" t="str">
@@ -8308,9 +8651,11 @@
       </x:c>
       <x:c r="M62" s="17" t="str"/>
       <x:c r="N62" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O62" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O62" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="42" customHeight="1">
       <x:c r="A63" s="17" t="str">
@@ -8349,9 +8694,11 @@
       </x:c>
       <x:c r="M63" s="17" t="str"/>
       <x:c r="N63" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O63" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O63" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="42" customHeight="1">
       <x:c r="A64" s="17" t="str">
@@ -8392,9 +8739,11 @@
         <x:v>[I-H-04] database snapshot is unchanged</x:v>
       </x:c>
       <x:c r="N64" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O64" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O64" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="42" customHeight="1">
       <x:c r="A65" s="17" t="str">
@@ -8433,25 +8782,28 @@
       </x:c>
       <x:c r="M65" s="17" t="str"/>
       <x:c r="N65" s="17" t="str">
-        <x:v>NO</x:v>
-      </x:c>
-      <x:c r="O65" s="17" t="str"/>
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="O65" s="17" t="str">
+        <x:v>Student personally reviewed all test-case rows on 2026-08-30.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="D5:D65">
-    <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="INVALID"/>
-    <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="INCOMPLETE"/>
-    <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="STUDENT_ADDED"/>
+    <x:cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="INVALID"/>
+    <x:cfRule type="containsText" dxfId="15" priority="2" operator="containsText" text="INCOMPLETE"/>
+    <x:cfRule type="containsText" dxfId="16" priority="3" operator="containsText" text="STUDENT_ADDED"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="L5:L65">
-    <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="PASS"/>
-    <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="FAIL"/>
+    <x:cfRule type="containsText" dxfId="17" priority="4" operator="containsText" text="PASS"/>
+    <x:cfRule type="containsText" dxfId="18" priority="5" operator="containsText" text="FAIL"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="N5:N65">
-    <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="NO"/>
+    <x:cfRule type="containsText" dxfId="19" priority="6" operator="containsText" text="NO"/>
+    <x:cfRule type="containsText" dxfId="20" priority="7" operator="containsText" text="YES"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="N5:N65">
@@ -8460,7 +8812,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a2d259f3fc439e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e43bb951d8a4c8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8742,7 +9094,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8e67f7c060c4ee0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa3741dc2814aa5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9039,12 +9391,12 @@
     <x:mergeCell ref="A1:G2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B5:B14">
-    <x:cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="Critical"/>
-    <x:cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="High"/>
+    <x:cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="Critical"/>
+    <x:cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="High"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7319e86383fd424a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22405c8fab934542"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9122,7 +9474,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str">
         <x:v>Student</x:v>
@@ -9139,7 +9491,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E7" s="16" t="str">
         <x:v>Student</x:v>
@@ -9224,7 +9576,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D12" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
         <x:v>Student</x:v>
@@ -9303,8 +9655,8 @@
     <x:mergeCell ref="A1:E2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="D5:D16">
-    <x:cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="NO"/>
-    <x:cfRule type="containsText" dxfId="24" priority="2" operator="containsText" text="YES"/>
+    <x:cfRule type="containsText" dxfId="26" priority="1" operator="containsText" text="NO"/>
+    <x:cfRule type="containsText" dxfId="27" priority="2" operator="containsText" text="YES"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="D5:D16">
@@ -9313,7 +9665,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47ce4670b2b54e01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R661a527cc2664baf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record final review and public repository
</commit_message>
<xml_diff>
--- a/outputs/hw06/HW06_Test_Cases.xlsx
+++ b/outputs/hw06/HW06_Test_Cases.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra2ff1d76981a4844"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="R340518ee2fba4600"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="R44810980d808440b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="Rc7f8c0b94bff4249"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="R8c6034ad32964dc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="R8fa87e8b6f35443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="Re128b7480cb94576"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc2312a2b87684351"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset_Password" sheetId="2" r:id="Ra3dec8c7e99f43c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apply_Coupon" sheetId="3" r:id="Rc803030aefc94953"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_Products" sheetId="4" r:id="R410c34c3da83476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Audit_Index" sheetId="5" r:id="R7bc91a01cf6d408c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug_Summary" sheetId="6" r:id="R7da503dc44d14cbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Review" sheetId="7" r:id="R9ee7a075f40b40d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -716,7 +716,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R29e19f29abb64de4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf359875259c54eec"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1400,7 +1400,7 @@
         <x:v>Public GitHub</x:v>
       </x:c>
       <x:c r="B17" s="42" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="C17" s="37"/>
       <x:c r="D17" s="37"/>
@@ -1513,7 +1513,7 @@
     <x:cfRule type="containsText" dxfId="23" priority="3" operator="containsText" text="/100"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8930911bef34d5d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4437ac4cdb54a2a"/>
 </x:worksheet>
 </file>
 
@@ -3744,7 +3744,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R563776ffe5e14c1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5af7e642e321499e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6013,7 +6013,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43aab7efe078463a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e1d3ad4618f4f40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8812,7 +8812,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e43bb951d8a4c8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R943fc59b52b2402e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9094,7 +9094,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aa3741dc2814aa5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b530b9a5421472e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9396,7 +9396,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22405c8fab934542"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2277e7b5609e4f5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9508,7 +9508,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str">
         <x:v>Student</x:v>
@@ -9525,7 +9525,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
         <x:v>Student</x:v>
@@ -9593,7 +9593,7 @@
         <x:v>BLOCKING</x:v>
       </x:c>
       <x:c r="D13" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
         <x:v>Student</x:v>
@@ -9665,7 +9665,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R661a527cc2664baf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd46447b93ae94455"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>